<commit_message>
Complete StageMesh identity migration
</commit_message>
<xml_diff>
--- a/docs/backlog/StageMesh-Master-Backlog-Refresh-2026-10-03.xlsx
+++ b/docs/backlog/StageMesh-Master-Backlog-Refresh-2026-10-03.xlsx
@@ -1665,7 +1665,7 @@
         <x:v>REC-033, WIT-048</x:v>
       </x:c>
       <x:c r="K3" s="15" t="str">
-        <x:v>No StageForge node, shared host, shared power/network failure domain or single witness can unilaterally authorize recovery</x:v>
+        <x:v>No StageMesh node, shared host, shared power/network failure domain or single witness can unilaterally authorize recovery</x:v>
       </x:c>
       <x:c r="L3" s="15" t="str">
         <x:v>Independent witness host/network/power failure-domain exercise</x:v>
@@ -1695,7 +1695,7 @@
         <x:v>Proxy-HTTPS deployment contract + qualification tooling</x:v>
       </x:c>
       <x:c r="E4" s="15" t="str">
-        <x:v>Make the reviewed TLS/auth reverse-proxy boundary machine-checkable while keeping the StageForge backend loopback-only</x:v>
+        <x:v>Make the reviewed TLS/auth reverse-proxy boundary machine-checkable while keeping the StageMesh backend loopback-only</x:v>
       </x:c>
       <x:c r="F4" s="15" t="str">
         <x:v>P0</x:v>
@@ -2961,10 +2961,10 @@
         <x:v>PKG-033, Checkpoint 68 device-permission verifier</x:v>
       </x:c>
       <x:c r="K30" s="15" t="str">
-        <x:v>The stageforge service identity has only the documented read/write access to required character-device nodes; symlink/non-device paths fail closed and no installer step broadens host permissions automatically</x:v>
+        <x:v>The stagemesh service identity has only the documented read/write access to required character-device nodes; symlink/non-device paths fail closed and no installer step broadens host permissions automatically</x:v>
       </x:c>
       <x:c r="L30" s="15" t="str">
-        <x:v>Clean-host run as stageforge using stageforge-device-permissions.py plus service/udev/group evidence</x:v>
+        <x:v>Clean-host run as stagemesh using stagemesh-device-permissions.py plus service/udev/group evidence</x:v>
       </x:c>
       <x:c r="M30" s="15" t="str">
         <x:v>Critical</x:v>
@@ -5247,7 +5247,7 @@
         <x:v>2/2 RT native CTest</x:v>
       </x:c>
       <x:c r="F48" t="str">
-        <x:v>Real clean-host stageforge-user ALSA/MIDI/UWB device permission matrix</x:v>
+        <x:v>Real clean-host stagemesh-user ALSA/MIDI/UWB device permission matrix</x:v>
       </x:c>
       <x:c r="G48" t="str">
         <x:v>2026-09-14</x:v>
@@ -5356,7 +5356,7 @@
         <x:v>654</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Generic CI + StageForge Platform Modules green; Windows and Apple Silicon native-launch artifacts qualified</x:v>
+        <x:v>Generic CI + StageMesh Platform Modules green; Windows and Apple Silicon native-launch artifacts qualified</x:v>
       </x:c>
       <x:c r="E53" t="str">
         <x:v>Checkpoint 69 local 2/2 RT native CTest baseline retained</x:v>
@@ -5881,7 +5881,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>Real clean-host/VM boot and upgrade exercise plus stageforge-user runs of the installed device-permission verifier against actual ALSA/MIDI/UWB nodes</x:v>
+        <x:v>Real clean-host/VM boot and upgrade exercise plus stagemesh-user runs of the installed device-permission verifier against actual ALSA/MIDI/UWB nodes</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
         <x:v>PKG-033, PKG-034</x:v>
@@ -6521,7 +6521,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="81" t="str">
-        <x:v>StageForge External Qualification Plan</x:v>
+        <x:v>StageMesh External Qualification Plan</x:v>
       </x:c>
       <x:c r="B1" s="81"/>
       <x:c r="C1" s="81"/>
@@ -6602,7 +6602,7 @@
         <x:v>three independently hosted witnesses plus primary/standby nodes</x:v>
       </x:c>
       <x:c r="D5" s="15" t="str">
-        <x:v>stageforge-witness-qualify.py</x:v>
+        <x:v>stagemesh-witness-qualify.py</x:v>
       </x:c>
       <x:c r="E5" s="15" t="str">
         <x:v>physicalIndependenceQualified
@@ -6640,7 +6640,7 @@
         <x:v>deployed TLS reverse proxy, IdP/auth proxy and venue/control LAN firewall</x:v>
       </x:c>
       <x:c r="D6" s="15" t="str">
-        <x:v>stageforge-http-qualify.py</x:v>
+        <x:v>stagemesh-http-qualify.py</x:v>
       </x:c>
       <x:c r="E6" s="15" t="str">
         <x:v>trustedCertificateQualified
@@ -6678,7 +6678,7 @@
         <x:v>fresh Linux host or VM with representative audio/MIDI/device access</x:v>
       </x:c>
       <x:c r="D7" s="15" t="str">
-        <x:v>stageforge-package-qualify.py</x:v>
+        <x:v>stagemesh-package-qualify.py</x:v>
       </x:c>
       <x:c r="E7" s="15" t="str">
         <x:v>cleanHostQualified
@@ -6862,7 +6862,7 @@
         <x:v>named production hardware and rehearsal topology</x:v>
       </x:c>
       <x:c r="D12" s="15" t="str">
-        <x:v>stageforge-qualify.py</x:v>
+        <x:v>stagemesh-qualify.py</x:v>
       </x:c>
       <x:c r="E12" s="15" t="str">
         <x:v>latencySoakQualified
@@ -6993,7 +6993,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="100" t="str">
-        <x:v>StageForge Qualification Intake Status</x:v>
+        <x:v>StageMesh Qualification Intake Status</x:v>
       </x:c>
       <x:c r="B1" s="100"/>
       <x:c r="C1" s="100"/>
@@ -7306,7 +7306,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="111" t="str">
-        <x:v>StageForge CI Platform Evidence</x:v>
+        <x:v>StageMesh CI Platform Evidence</x:v>
       </x:c>
       <x:c r="B1" s="111"/>
       <x:c r="C1" s="111"/>
@@ -7452,7 +7452,7 @@
         <x:v>Not claimed</x:v>
       </x:c>
       <x:c r="G8" s="12" t="str">
-        <x:v>https://github.com/colinatwood/stageforge/actions/runs/34998947927
+        <x:v>https://github.com/colinatwood/stagemesh/actions/runs/34998947927
 Selected-loss binary SHA-256: 7dfd0ae3c4e3351535f88616a560ef103bb8977137e83cb23cd310f1b8f4cebd</x:v>
       </x:c>
       <x:c r="H8" s="12" t="str">
@@ -7479,7 +7479,7 @@
         <x:v>Not claimed</x:v>
       </x:c>
       <x:c r="G9" s="12" t="str">
-        <x:v>https://github.com/colinatwood/stageforge/actions/runs/34998947927
+        <x:v>https://github.com/colinatwood/stagemesh/actions/runs/34998947927
 Selected-loss binary SHA-256: 2b6ed39303c309e52150c0abc0600fe052c37502d3f44506ffc99319d44502d9</x:v>
       </x:c>
       <x:c r="H9" s="12" t="str">

</xml_diff>

<commit_message>
Complete StageMesh identity migration (#91)
Remove the retired product identity across source, packaging, runtime contracts, documentation, and backlog artifacts. Add a repository-wide regression guard while preserving external qualification boundaries.
</commit_message>
<xml_diff>
--- a/docs/backlog/StageMesh-Master-Backlog-Refresh-2026-10-03.xlsx
+++ b/docs/backlog/StageMesh-Master-Backlog-Refresh-2026-10-03.xlsx
@@ -1665,7 +1665,7 @@
         <x:v>REC-033, WIT-048</x:v>
       </x:c>
       <x:c r="K3" s="15" t="str">
-        <x:v>No StageForge node, shared host, shared power/network failure domain or single witness can unilaterally authorize recovery</x:v>
+        <x:v>No StageMesh node, shared host, shared power/network failure domain or single witness can unilaterally authorize recovery</x:v>
       </x:c>
       <x:c r="L3" s="15" t="str">
         <x:v>Independent witness host/network/power failure-domain exercise</x:v>
@@ -1695,7 +1695,7 @@
         <x:v>Proxy-HTTPS deployment contract + qualification tooling</x:v>
       </x:c>
       <x:c r="E4" s="15" t="str">
-        <x:v>Make the reviewed TLS/auth reverse-proxy boundary machine-checkable while keeping the StageForge backend loopback-only</x:v>
+        <x:v>Make the reviewed TLS/auth reverse-proxy boundary machine-checkable while keeping the StageMesh backend loopback-only</x:v>
       </x:c>
       <x:c r="F4" s="15" t="str">
         <x:v>P0</x:v>
@@ -2961,10 +2961,10 @@
         <x:v>PKG-033, Checkpoint 68 device-permission verifier</x:v>
       </x:c>
       <x:c r="K30" s="15" t="str">
-        <x:v>The stageforge service identity has only the documented read/write access to required character-device nodes; symlink/non-device paths fail closed and no installer step broadens host permissions automatically</x:v>
+        <x:v>The stagemesh service identity has only the documented read/write access to required character-device nodes; symlink/non-device paths fail closed and no installer step broadens host permissions automatically</x:v>
       </x:c>
       <x:c r="L30" s="15" t="str">
-        <x:v>Clean-host run as stageforge using stageforge-device-permissions.py plus service/udev/group evidence</x:v>
+        <x:v>Clean-host run as stagemesh using stagemesh-device-permissions.py plus service/udev/group evidence</x:v>
       </x:c>
       <x:c r="M30" s="15" t="str">
         <x:v>Critical</x:v>
@@ -5247,7 +5247,7 @@
         <x:v>2/2 RT native CTest</x:v>
       </x:c>
       <x:c r="F48" t="str">
-        <x:v>Real clean-host stageforge-user ALSA/MIDI/UWB device permission matrix</x:v>
+        <x:v>Real clean-host stagemesh-user ALSA/MIDI/UWB device permission matrix</x:v>
       </x:c>
       <x:c r="G48" t="str">
         <x:v>2026-09-14</x:v>
@@ -5356,7 +5356,7 @@
         <x:v>654</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Generic CI + StageForge Platform Modules green; Windows and Apple Silicon native-launch artifacts qualified</x:v>
+        <x:v>Generic CI + StageMesh Platform Modules green; Windows and Apple Silicon native-launch artifacts qualified</x:v>
       </x:c>
       <x:c r="E53" t="str">
         <x:v>Checkpoint 69 local 2/2 RT native CTest baseline retained</x:v>
@@ -5881,7 +5881,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>Real clean-host/VM boot and upgrade exercise plus stageforge-user runs of the installed device-permission verifier against actual ALSA/MIDI/UWB nodes</x:v>
+        <x:v>Real clean-host/VM boot and upgrade exercise plus stagemesh-user runs of the installed device-permission verifier against actual ALSA/MIDI/UWB nodes</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
         <x:v>PKG-033, PKG-034</x:v>
@@ -6521,7 +6521,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="81" t="str">
-        <x:v>StageForge External Qualification Plan</x:v>
+        <x:v>StageMesh External Qualification Plan</x:v>
       </x:c>
       <x:c r="B1" s="81"/>
       <x:c r="C1" s="81"/>
@@ -6602,7 +6602,7 @@
         <x:v>three independently hosted witnesses plus primary/standby nodes</x:v>
       </x:c>
       <x:c r="D5" s="15" t="str">
-        <x:v>stageforge-witness-qualify.py</x:v>
+        <x:v>stagemesh-witness-qualify.py</x:v>
       </x:c>
       <x:c r="E5" s="15" t="str">
         <x:v>physicalIndependenceQualified
@@ -6640,7 +6640,7 @@
         <x:v>deployed TLS reverse proxy, IdP/auth proxy and venue/control LAN firewall</x:v>
       </x:c>
       <x:c r="D6" s="15" t="str">
-        <x:v>stageforge-http-qualify.py</x:v>
+        <x:v>stagemesh-http-qualify.py</x:v>
       </x:c>
       <x:c r="E6" s="15" t="str">
         <x:v>trustedCertificateQualified
@@ -6678,7 +6678,7 @@
         <x:v>fresh Linux host or VM with representative audio/MIDI/device access</x:v>
       </x:c>
       <x:c r="D7" s="15" t="str">
-        <x:v>stageforge-package-qualify.py</x:v>
+        <x:v>stagemesh-package-qualify.py</x:v>
       </x:c>
       <x:c r="E7" s="15" t="str">
         <x:v>cleanHostQualified
@@ -6862,7 +6862,7 @@
         <x:v>named production hardware and rehearsal topology</x:v>
       </x:c>
       <x:c r="D12" s="15" t="str">
-        <x:v>stageforge-qualify.py</x:v>
+        <x:v>stagemesh-qualify.py</x:v>
       </x:c>
       <x:c r="E12" s="15" t="str">
         <x:v>latencySoakQualified
@@ -6993,7 +6993,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="100" t="str">
-        <x:v>StageForge Qualification Intake Status</x:v>
+        <x:v>StageMesh Qualification Intake Status</x:v>
       </x:c>
       <x:c r="B1" s="100"/>
       <x:c r="C1" s="100"/>
@@ -7306,7 +7306,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="111" t="str">
-        <x:v>StageForge CI Platform Evidence</x:v>
+        <x:v>StageMesh CI Platform Evidence</x:v>
       </x:c>
       <x:c r="B1" s="111"/>
       <x:c r="C1" s="111"/>
@@ -7452,7 +7452,7 @@
         <x:v>Not claimed</x:v>
       </x:c>
       <x:c r="G8" s="12" t="str">
-        <x:v>https://github.com/colinatwood/stageforge/actions/runs/34998947927
+        <x:v>https://github.com/colinatwood/stagemesh/actions/runs/34998947927
 Selected-loss binary SHA-256: 7dfd0ae3c4e3351535f88616a560ef103bb8977137e83cb23cd310f1b8f4cebd</x:v>
       </x:c>
       <x:c r="H8" s="12" t="str">
@@ -7479,7 +7479,7 @@
         <x:v>Not claimed</x:v>
       </x:c>
       <x:c r="G9" s="12" t="str">
-        <x:v>https://github.com/colinatwood/stageforge/actions/runs/34998947927
+        <x:v>https://github.com/colinatwood/stagemesh/actions/runs/34998947927
 Selected-loss binary SHA-256: 2b6ed39303c309e52150c0abc0600fe052c37502d3f44506ffc99319d44502d9</x:v>
       </x:c>
       <x:c r="H9" s="12" t="str">

</xml_diff>